<commit_message>
Update Quick Switcher Login, roles mapping, and real Excel testing data seeder (@elvith.id domain)
</commit_message>
<xml_diff>
--- a/Hasil_Setup_Santri_Wali_KomplekCD.xlsx
+++ b/Hasil_Setup_Santri_Wali_KomplekCD.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ambisss\My Projek Laravel\elf_v1\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A157B5C-3E13-4CDA-A7EA-1EDB3350D78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Isian Data Santri" sheetId="1" r:id="rId4"/>
+    <sheet name="Isian Data Santri" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="193">
   <si>
     <t>Nama Lengkap Santri *</t>
   </si>
@@ -594,37 +599,20 @@
   </si>
   <si>
     <t>otomotif (kerja)</t>
-  </si>
-  <si>
-    <t>Yusuf Ali(boyong tanpa diketahui)</t>
-  </si>
-  <si>
-    <t>Kamar Umum</t>
-  </si>
-  <si>
-    <t>awan (boyong tanpa diketahui)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
@@ -657,14 +645,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -954,31 +950,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:O41"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O39"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.99" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="4.57" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="4.57" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="32.992" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="35.277" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="67.127" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="40" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="35.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="67.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1025,7 +1017,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1057,7 +1049,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1092,7 +1084,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1124,7 +1116,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -1159,7 +1151,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -1194,7 +1186,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -1229,7 +1221,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -1264,7 +1256,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -1299,7 +1291,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -1334,7 +1326,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -1369,7 +1361,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>71</v>
       </c>
@@ -1404,7 +1396,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>75</v>
       </c>
@@ -1439,7 +1431,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>79</v>
       </c>
@@ -1474,7 +1466,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>85</v>
       </c>
@@ -1506,7 +1498,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -1538,7 +1530,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -1573,7 +1565,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>100</v>
       </c>
@@ -1608,7 +1600,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>103</v>
       </c>
@@ -1643,7 +1635,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>108</v>
       </c>
@@ -1678,7 +1670,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>112</v>
       </c>
@@ -1713,7 +1705,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>119</v>
       </c>
@@ -1748,7 +1740,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>124</v>
       </c>
@@ -1783,7 +1775,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>129</v>
       </c>
@@ -1818,7 +1810,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>134</v>
       </c>
@@ -1853,7 +1845,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>138</v>
       </c>
@@ -1888,7 +1880,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>143</v>
       </c>
@@ -1923,7 +1915,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>147</v>
       </c>
@@ -1958,7 +1950,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>152</v>
       </c>
@@ -1993,7 +1985,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>155</v>
       </c>
@@ -2028,7 +2020,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>158</v>
       </c>
@@ -2063,7 +2055,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>162</v>
       </c>
@@ -2098,7 +2090,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>166</v>
       </c>
@@ -2133,7 +2125,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>171</v>
       </c>
@@ -2168,7 +2160,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>175</v>
       </c>
@@ -2203,7 +2195,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>180</v>
       </c>
@@ -2238,7 +2230,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>184</v>
       </c>
@@ -2273,7 +2265,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>188</v>
       </c>
@@ -2308,7 +2300,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>191</v>
       </c>
@@ -2340,70 +2332,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="40" spans="1:15">
-      <c r="A40" t="s">
-        <v>193</v>
-      </c>
-      <c r="D40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" t="s">
-        <v>17</v>
-      </c>
-      <c r="H40" t="s">
-        <v>113</v>
-      </c>
-      <c r="I40" t="s">
-        <v>194</v>
-      </c>
-      <c r="K40" t="s">
-        <v>130</v>
-      </c>
-      <c r="L40" t="s">
-        <v>22</v>
-      </c>
-      <c r="M40" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15">
-      <c r="A41" t="s">
-        <v>195</v>
-      </c>
-      <c r="D41" t="s">
-        <v>16</v>
-      </c>
-      <c r="G41" t="s">
-        <v>17</v>
-      </c>
-      <c r="H41" t="s">
-        <v>113</v>
-      </c>
-      <c r="I41" t="s">
-        <v>194</v>
-      </c>
-      <c r="K41" t="s">
-        <v>130</v>
-      </c>
-      <c r="L41" t="s">
-        <v>22</v>
-      </c>
-      <c r="M41" t="s">
-        <v>23</v>
-      </c>
-    </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>